<commit_message>
fix(onboarding): PUNTO 7 · inversiones cierra el bucle + plantilla espejo
- P1: la vía "una a una" abre /inversiones?from=empezar; la galería abre el
  selector directo y vuelve al flujo al crear (o cancelar). Importadores de
  broker (Indexa · Aportaciones CSV) propagan from=empezar y vuelven con ?done.
- P2: syncNucleoFromData marca el bloque inversiones (store inversiones +
  planesPensiones) → crear posición sube el %.
- P3: plantilla espejo de las 6 familias (plan_pensiones/fondo/accion_etf_reit/
  prestamo_activo/deposito_cuenta/crypto) con subtipo · ISIN · % atribución ·
  TAE · plazo como opcionales. Parser resuelve columnas por nombre (plantilla
  vieja de 7 columnas sigue funcionando). Fechas DD/MM/AAAA.
- P4: préstamo-activo (te deben) → store inversiones, nunca al store prestamos.
</commit_message>
<xml_diff>
--- a/public/templates/plantilla-inversiones-atlas.xlsx
+++ b/public/templates/plantilla-inversiones-atlas.xlsx
@@ -4,6 +4,7 @@
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
     <sheet name="Atlas" sheetId="1" r:id="rId1"/>
+    <sheet name="Léeme" sheetId="2" r:id="rId2"/>
   </sheets>
 </workbook>
 </file>
@@ -399,57 +400,391 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:L8"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Tipo (fondo/accion/etf/crypto/plan_pensiones/deposito/otro)</v>
+        <v>Tipo (plan_pensiones/fondo/accion_etf_reit/prestamo_activo/deposito_cuenta/crypto)</v>
       </c>
       <c r="B1" t="str">
+        <v>Subtipo (PPE·PPI · accion·ETF·REIT · P2P·empresa · plazo·cuenta)</v>
+      </c>
+      <c r="C1" t="str">
         <v>Entidad</v>
       </c>
-      <c r="C1" t="str">
+      <c r="D1" t="str">
         <v>Producto</v>
       </c>
-      <c r="D1" t="str">
-        <v>Unidades</v>
-      </c>
       <c r="E1" t="str">
+        <v>ISIN o ticker</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Unidades / participaciones</v>
+      </c>
+      <c r="G1" t="str">
         <v>Coste adquisición €</v>
       </c>
-      <c r="F1" t="str">
+      <c r="H1" t="str">
         <v>Fecha compra</v>
       </c>
-      <c r="G1" t="str">
+      <c r="I1" t="str">
         <v>Valor de hoy €</v>
+      </c>
+      <c r="J1" t="str">
+        <v>% atribución (participaciones)</v>
+      </c>
+      <c r="K1" t="str">
+        <v>TAE/TIN %</v>
+      </c>
+      <c r="L1" t="str">
+        <v>Plazo (meses)</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
+        <v>plan_pensiones</v>
+      </c>
+      <c r="B2" t="str">
+        <v>PPE</v>
+      </c>
+      <c r="C2" t="str">
+        <v>VidaCaixa</v>
+      </c>
+      <c r="D2" t="str">
+        <v>PPE Empresa</v>
+      </c>
+      <c r="E2" t="str">
+        <v/>
+      </c>
+      <c r="F2" t="str">
+        <v/>
+      </c>
+      <c r="G2">
+        <v>8000</v>
+      </c>
+      <c r="H2" s="1">
+        <v>43845</v>
+      </c>
+      <c r="I2">
+        <v>9200</v>
+      </c>
+      <c r="J2" t="str">
+        <v/>
+      </c>
+      <c r="K2" t="str">
+        <v/>
+      </c>
+      <c r="L2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
         <v>fondo</v>
       </c>
-      <c r="B2" t="str">
+      <c r="B3" t="str">
+        <v>FI</v>
+      </c>
+      <c r="C3" t="str">
         <v>Indexa Capital</v>
       </c>
-      <c r="C2" t="str">
+      <c r="D3" t="str">
         <v>Indexa RV Mixta</v>
       </c>
-      <c r="D2">
+      <c r="E3" t="str">
+        <v>IE00B4L5Y983</v>
+      </c>
+      <c r="F3">
         <v>120</v>
       </c>
-      <c r="E2">
+      <c r="G3">
         <v>10000</v>
       </c>
-      <c r="F2" s="1">
+      <c r="H3" s="1">
         <v>44630</v>
       </c>
-      <c r="G2">
+      <c r="I3">
         <v>12500</v>
+      </c>
+      <c r="J3" t="str">
+        <v/>
+      </c>
+      <c r="K3" t="str">
+        <v/>
+      </c>
+      <c r="L3" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>accion_etf_reit</v>
+      </c>
+      <c r="B4" t="str">
+        <v>ETF</v>
+      </c>
+      <c r="C4" t="str">
+        <v>DEGIRO</v>
+      </c>
+      <c r="D4" t="str">
+        <v>iShares Core S&amp;P 500</v>
+      </c>
+      <c r="E4" t="str">
+        <v>IE00B5BMR087</v>
+      </c>
+      <c r="F4">
+        <v>50</v>
+      </c>
+      <c r="G4">
+        <v>18000</v>
+      </c>
+      <c r="H4" s="1">
+        <v>44440</v>
+      </c>
+      <c r="I4">
+        <v>24500</v>
+      </c>
+      <c r="J4" t="str">
+        <v/>
+      </c>
+      <c r="K4" t="str">
+        <v/>
+      </c>
+      <c r="L4" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>accion_etf_reit</v>
+      </c>
+      <c r="B5" t="str">
+        <v>accion</v>
+      </c>
+      <c r="C5" t="str">
+        <v>CB Hermanos</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Participación CB</v>
+      </c>
+      <c r="E5" t="str">
+        <v/>
+      </c>
+      <c r="F5">
+        <v>1</v>
+      </c>
+      <c r="G5">
+        <v>30000</v>
+      </c>
+      <c r="H5" s="1">
+        <v>43617</v>
+      </c>
+      <c r="I5">
+        <v>35000</v>
+      </c>
+      <c r="J5">
+        <v>33.34</v>
+      </c>
+      <c r="K5" t="str">
+        <v/>
+      </c>
+      <c r="L5" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>prestamo_activo</v>
+      </c>
+      <c r="B6" t="str">
+        <v>P2P</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Mintos</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Préstamo SmartFlip</v>
+      </c>
+      <c r="E6" t="str">
+        <v/>
+      </c>
+      <c r="F6" t="str">
+        <v/>
+      </c>
+      <c r="G6">
+        <v>5000</v>
+      </c>
+      <c r="H6" s="1">
+        <v>44936</v>
+      </c>
+      <c r="I6">
+        <v>5000</v>
+      </c>
+      <c r="J6" t="str">
+        <v/>
+      </c>
+      <c r="K6">
+        <v>10</v>
+      </c>
+      <c r="L6">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>deposito_cuenta</v>
+      </c>
+      <c r="B7" t="str">
+        <v>plazo</v>
+      </c>
+      <c r="C7" t="str">
+        <v>EBN Banco</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Depósito 12 meses</v>
+      </c>
+      <c r="E7" t="str">
+        <v/>
+      </c>
+      <c r="F7" t="str">
+        <v/>
+      </c>
+      <c r="G7">
+        <v>20000</v>
+      </c>
+      <c r="H7" s="1">
+        <v>45352</v>
+      </c>
+      <c r="I7">
+        <v>20000</v>
+      </c>
+      <c r="J7" t="str">
+        <v/>
+      </c>
+      <c r="K7">
+        <v>3.2</v>
+      </c>
+      <c r="L7">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>crypto</v>
+      </c>
+      <c r="B8" t="str">
+        <v/>
+      </c>
+      <c r="C8" t="str">
+        <v>Kraken</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Bitcoin</v>
+      </c>
+      <c r="E8" t="str">
+        <v/>
+      </c>
+      <c r="F8">
+        <v>0.5</v>
+      </c>
+      <c r="G8">
+        <v>15000</v>
+      </c>
+      <c r="H8" s="1">
+        <v>44505</v>
+      </c>
+      <c r="I8">
+        <v>22000</v>
+      </c>
+      <c r="J8" t="str">
+        <v/>
+      </c>
+      <c r="K8" t="str">
+        <v/>
+      </c>
+      <c r="L8" t="str">
+        <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L8"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:A13"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>PLANTILLA DE INVERSIONES · Atlas</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Obligatorias: Tipo y Producto. El resto es opcional; lo que dejes vacío</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>lo podrás completar luego en la ficha de la posición.</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Tipo (familia): plan_pensiones · fondo · accion_etf_reit · prestamo_activo ·</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>deposito_cuenta · crypto. El Subtipo afina la clase (PPE, ETF, REIT, P2P,</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>cuenta, plazo…).</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>Préstamo_activo = dinero que TE DEBEN (P2P o a empresa) · NO es tu hipoteca</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>(esa va en el bloque Préstamos).</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>Fechas en formato DD/MM/AAAA. Importes con coma decimal (1.234,56).</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:A13"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>